<commit_message>
Update WDATA Forwarding Unit
</commit_message>
<xml_diff>
--- a/document/IDD.xlsx
+++ b/document/IDD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\SoC_Design\document\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D16C1C-4E28-4F74-A8C8-EA60B194CC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B2EBC6C-9D03-459A-8574-BF7AC61684FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="380">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="631" uniqueCount="381">
   <si>
     <t>Signal</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -295,11 +295,6 @@
   </si>
   <si>
     <t>-</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>o_d_mem_en
-o_d_mem_wren</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -1575,6 +1570,39 @@
 u_wdata_forwarding_unit
 u_alu_forwarding_unit
 u_jump_forwarding_unit</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>u_wdata_forwarding_unit</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+o_d_mem_en
+o_d_mem_wren</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>u_ex_mem_bridge
+u_wdata_forwarding_unit</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2828,7 +2856,7 @@
     <row r="1" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B2" s="129" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C2" s="130"/>
       <c r="D2" s="130"/>
@@ -3061,10 +3089,10 @@
         <v>11</v>
       </c>
       <c r="C14" s="51" t="s">
+        <v>254</v>
+      </c>
+      <c r="D14" s="37" t="s">
         <v>255</v>
-      </c>
-      <c r="D14" s="37" t="s">
-        <v>256</v>
       </c>
       <c r="E14" s="53" t="s">
         <v>22</v>
@@ -3119,7 +3147,7 @@
     <row r="17" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="2:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="132" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C18" s="133"/>
       <c r="D18" s="133"/>
@@ -3153,19 +3181,19 @@
         <v>1</v>
       </c>
       <c r="C20" s="103" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D20" s="104">
         <v>1</v>
       </c>
       <c r="E20" s="103" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F20" s="128" t="s">
         <v>63</v>
       </c>
       <c r="G20" s="105" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3174,19 +3202,19 @@
         <v>2</v>
       </c>
       <c r="C21" s="57" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D21" s="58">
         <v>4</v>
       </c>
       <c r="E21" s="57" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F21" s="71" t="s">
+        <v>64</v>
+      </c>
+      <c r="G21" s="90" t="s">
         <v>65</v>
-      </c>
-      <c r="G21" s="90" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3195,19 +3223,19 @@
         <v>3</v>
       </c>
       <c r="C22" s="57" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="D22" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E22" s="57" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F22" s="71" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G22" s="90" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.3">
@@ -3216,19 +3244,19 @@
         <v>4</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D23" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E23" s="57" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F23" s="71" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G23" s="90" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -3237,19 +3265,19 @@
         <v>5</v>
       </c>
       <c r="C24" s="57" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D24" s="58">
         <v>1</v>
       </c>
       <c r="E24" s="57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F24" s="71" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G24" s="90" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="25" spans="2:7" x14ac:dyDescent="0.3">
@@ -3258,19 +3286,19 @@
         <v>6</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D25" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E25" s="57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F25" s="71" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G25" s="90" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="26" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3279,19 +3307,19 @@
         <v>7</v>
       </c>
       <c r="C26" s="57" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D26" s="58">
         <v>1</v>
       </c>
       <c r="E26" s="57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F26" s="71" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G26" s="90" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="27" spans="2:7" x14ac:dyDescent="0.3">
@@ -3300,19 +3328,19 @@
         <v>8</v>
       </c>
       <c r="C27" s="57" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D27" s="58">
         <v>4</v>
       </c>
       <c r="E27" s="57" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F27" s="59" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G27" s="90" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3321,19 +3349,19 @@
         <v>9</v>
       </c>
       <c r="C28" s="57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D28" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E28" s="57" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F28" s="71" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G28" s="90" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.3">
@@ -3342,19 +3370,19 @@
         <v>10</v>
       </c>
       <c r="C29" s="57" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D29" s="73" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E29" s="74" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F29" s="71" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G29" s="97" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="30" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3363,19 +3391,19 @@
         <v>11</v>
       </c>
       <c r="C30" s="72" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D30" s="58" t="s">
+        <v>286</v>
+      </c>
+      <c r="E30" s="74" t="s">
         <v>287</v>
       </c>
-      <c r="E30" s="74" t="s">
+      <c r="F30" s="74" t="s">
         <v>288</v>
       </c>
-      <c r="F30" s="74" t="s">
-        <v>289</v>
-      </c>
       <c r="G30" s="98" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="31" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3384,19 +3412,19 @@
         <v>12</v>
       </c>
       <c r="C31" s="72" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D31" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E31" s="74" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F31" s="74" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G31" s="98" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="32" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3405,19 +3433,19 @@
         <v>13</v>
       </c>
       <c r="C32" s="72" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D32" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E32" s="74" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F32" s="74" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G32" s="98" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3426,19 +3454,19 @@
         <v>14</v>
       </c>
       <c r="C33" s="72" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D33" s="58" t="s">
+        <v>286</v>
+      </c>
+      <c r="E33" s="74" t="s">
         <v>287</v>
       </c>
-      <c r="E33" s="74" t="s">
+      <c r="F33" s="74" t="s">
         <v>288</v>
       </c>
-      <c r="F33" s="74" t="s">
-        <v>289</v>
-      </c>
       <c r="G33" s="98" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
@@ -3447,19 +3475,19 @@
         <v>15</v>
       </c>
       <c r="C34" s="57" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D34" s="58">
         <v>3</v>
       </c>
       <c r="E34" s="59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F34" s="71" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="G34" s="90" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.3">
@@ -3468,7 +3496,7 @@
         <v>16</v>
       </c>
       <c r="C35" s="57" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D35" s="55" t="s">
         <v>19</v>
@@ -3480,7 +3508,7 @@
         <v>52</v>
       </c>
       <c r="G35" s="90" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="36" spans="2:7" x14ac:dyDescent="0.3">
@@ -3489,7 +3517,7 @@
         <v>17</v>
       </c>
       <c r="C36" s="57" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D36" s="55" t="s">
         <v>20</v>
@@ -3501,7 +3529,7 @@
         <v>35</v>
       </c>
       <c r="G36" s="90" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.3">
@@ -3510,19 +3538,19 @@
         <v>18</v>
       </c>
       <c r="C37" s="57" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D37" s="58">
         <v>1</v>
       </c>
       <c r="E37" s="57" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F37" s="59" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G37" s="90" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="2:7" ht="66" x14ac:dyDescent="0.3">
@@ -3531,19 +3559,19 @@
         <v>19</v>
       </c>
       <c r="C38" s="57" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D38" s="58">
         <v>1</v>
       </c>
       <c r="E38" s="71" t="s">
+        <v>330</v>
+      </c>
+      <c r="F38" s="71" t="s">
         <v>331</v>
       </c>
-      <c r="F38" s="71" t="s">
+      <c r="G38" s="90" t="s">
         <v>332</v>
-      </c>
-      <c r="G38" s="90" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="39" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -3552,19 +3580,19 @@
         <v>20</v>
       </c>
       <c r="C39" s="57" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D39" s="58">
         <v>1</v>
       </c>
       <c r="E39" s="74" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="F39" s="71" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G39" s="90" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="2:7" ht="66" x14ac:dyDescent="0.3">
@@ -3573,19 +3601,19 @@
         <v>21</v>
       </c>
       <c r="C40" s="57" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D40" s="58">
         <v>2</v>
       </c>
       <c r="E40" s="59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F40" s="71" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="G40" s="90" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.3">
@@ -3594,19 +3622,19 @@
         <v>22</v>
       </c>
       <c r="C41" s="57" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D41" s="58">
         <v>6</v>
       </c>
       <c r="E41" s="57" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F41" s="59" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G41" s="90" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="42" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3615,19 +3643,19 @@
         <v>23</v>
       </c>
       <c r="C42" s="57" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D42" s="55" t="s">
         <v>55</v>
       </c>
       <c r="E42" s="57" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F42" s="71" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="G42" s="90" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="43" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -3636,19 +3664,19 @@
         <v>24</v>
       </c>
       <c r="C43" s="57" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D43" s="55" t="s">
         <v>55</v>
       </c>
       <c r="E43" s="57" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F43" s="71" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="G43" s="90" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="44" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3657,19 +3685,19 @@
         <v>25</v>
       </c>
       <c r="C44" s="57" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D44" s="58">
         <v>1</v>
       </c>
       <c r="E44" s="74" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F44" s="71" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="G44" s="90" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.3">
@@ -3678,19 +3706,19 @@
         <v>26</v>
       </c>
       <c r="C45" s="57" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D45" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E45" s="57" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F45" s="59" t="s">
         <v>63</v>
       </c>
       <c r="G45" s="90" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.3">
@@ -3699,19 +3727,19 @@
         <v>27</v>
       </c>
       <c r="C46" s="57" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D46" s="60" t="s">
         <v>19</v>
       </c>
       <c r="E46" s="74" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F46" s="59" t="s">
         <v>35</v>
       </c>
       <c r="G46" s="90" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.3">
@@ -3720,7 +3748,7 @@
         <v>28</v>
       </c>
       <c r="C47" s="61" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D47" s="55" t="s">
         <v>20</v>
@@ -3729,10 +3757,10 @@
         <v>35</v>
       </c>
       <c r="F47" s="78" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G47" s="91" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="48" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3741,19 +3769,19 @@
         <v>29</v>
       </c>
       <c r="C48" s="72" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D48" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E48" s="74" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F48" s="74" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G48" s="98" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.3">
@@ -3762,19 +3790,19 @@
         <v>30</v>
       </c>
       <c r="C49" s="57" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D49" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E49" s="57" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F49" s="59" t="s">
         <v>63</v>
       </c>
       <c r="G49" s="90" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.3">
@@ -3783,19 +3811,19 @@
         <v>31</v>
       </c>
       <c r="C50" s="72" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D50" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E50" s="74" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F50" s="74" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G50" s="98" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="51" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3804,19 +3832,19 @@
         <v>32</v>
       </c>
       <c r="C51" s="57" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D51" s="58">
         <v>1</v>
       </c>
       <c r="E51" s="62" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F51" s="78" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G51" s="90" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.3">
@@ -3825,19 +3853,19 @@
         <v>33</v>
       </c>
       <c r="C52" s="72" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D52" s="55" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E52" s="74" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F52" s="74" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G52" s="98" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.3">
@@ -3846,40 +3874,40 @@
         <v>34</v>
       </c>
       <c r="C53" s="57" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D53" s="58">
         <v>1</v>
       </c>
       <c r="E53" s="59" t="s">
+        <v>117</v>
+      </c>
+      <c r="F53" s="71" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="71" t="s">
-        <v>119</v>
-      </c>
       <c r="G53" s="90" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="54" spans="2:7" x14ac:dyDescent="0.3">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" ht="33" x14ac:dyDescent="0.3">
       <c r="B54" s="89">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="C54" s="57" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D54" s="58">
         <v>1</v>
       </c>
       <c r="E54" s="62" t="s">
-        <v>118</v>
-      </c>
-      <c r="F54" s="62" t="s">
-        <v>119</v>
+        <v>117</v>
+      </c>
+      <c r="F54" s="78" t="s">
+        <v>380</v>
       </c>
       <c r="G54" s="90" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.3">
@@ -3888,19 +3916,19 @@
         <v>36</v>
       </c>
       <c r="C55" s="72" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D55" s="55" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E55" s="74" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F55" s="74" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G55" s="98" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="56" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -3909,19 +3937,19 @@
         <v>37</v>
       </c>
       <c r="C56" s="57" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D56" s="55" t="s">
         <v>20</v>
       </c>
       <c r="E56" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F56" s="71" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="G56" s="91" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="57" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3930,19 +3958,19 @@
         <v>38</v>
       </c>
       <c r="C57" s="57" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D57" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E57" s="57" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F57" s="71" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="G57" s="90" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="58" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -3951,19 +3979,19 @@
         <v>39</v>
       </c>
       <c r="C58" s="63" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D58" s="64" t="s">
         <v>19</v>
       </c>
       <c r="E58" s="63" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F58" s="79" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="G58" s="93" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="59" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -3972,19 +4000,19 @@
         <v>40</v>
       </c>
       <c r="C59" s="57" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D59" s="55" t="s">
         <v>55</v>
       </c>
       <c r="E59" s="57" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F59" s="71" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="G59" s="90" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.3">
@@ -3993,19 +4021,19 @@
         <v>41</v>
       </c>
       <c r="C60" s="57" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D60" s="58">
         <v>1</v>
       </c>
       <c r="E60" s="59" t="s">
+        <v>117</v>
+      </c>
+      <c r="F60" s="71" t="s">
         <v>118</v>
       </c>
-      <c r="F60" s="71" t="s">
-        <v>119</v>
-      </c>
       <c r="G60" s="90" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.3">
@@ -4014,7 +4042,7 @@
         <v>42</v>
       </c>
       <c r="C61" s="57" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D61" s="55" t="s">
         <v>48</v>
@@ -4023,7 +4051,7 @@
         <v>46</v>
       </c>
       <c r="F61" s="57" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G61" s="90" t="s">
         <v>53</v>
@@ -4035,13 +4063,13 @@
         <v>43</v>
       </c>
       <c r="C62" s="57" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D62" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E62" s="57" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F62" s="59" t="s">
         <v>39</v>
@@ -4056,19 +4084,19 @@
         <v>44</v>
       </c>
       <c r="C63" s="57" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D63" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E63" s="57" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F63" s="71" t="s">
         <v>47</v>
       </c>
       <c r="G63" s="90" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.3">
@@ -4077,19 +4105,19 @@
         <v>45</v>
       </c>
       <c r="C64" s="57" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D64" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E64" s="57" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F64" s="57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G64" s="90" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.3">
@@ -4098,19 +4126,19 @@
         <v>46</v>
       </c>
       <c r="C65" s="57" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D65" s="58">
         <v>1</v>
       </c>
       <c r="E65" s="59" t="s">
+        <v>211</v>
+      </c>
+      <c r="F65" s="59" t="s">
         <v>212</v>
       </c>
-      <c r="F65" s="59" t="s">
-        <v>213</v>
-      </c>
       <c r="G65" s="90" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.3">
@@ -4119,19 +4147,19 @@
         <v>47</v>
       </c>
       <c r="C66" s="57" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D66" s="58">
         <v>1</v>
       </c>
       <c r="E66" s="59" t="s">
+        <v>211</v>
+      </c>
+      <c r="F66" s="59" t="s">
         <v>212</v>
       </c>
-      <c r="F66" s="59" t="s">
-        <v>213</v>
-      </c>
       <c r="G66" s="90" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="67" spans="2:7" x14ac:dyDescent="0.3">
@@ -4140,19 +4168,19 @@
         <v>48</v>
       </c>
       <c r="C67" s="57" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D67" s="58">
         <v>1</v>
       </c>
       <c r="E67" s="59" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F67" s="59" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="G67" s="90" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="68" spans="2:7" x14ac:dyDescent="0.3">
@@ -4161,19 +4189,19 @@
         <v>49</v>
       </c>
       <c r="C68" s="57" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D68" s="58">
         <v>1</v>
       </c>
       <c r="E68" s="59" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F68" s="59" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G68" s="90" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.3">
@@ -4182,19 +4210,19 @@
         <v>50</v>
       </c>
       <c r="C69" s="57" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D69" s="58">
         <v>1</v>
       </c>
       <c r="E69" s="126" t="s">
+        <v>362</v>
+      </c>
+      <c r="F69" s="126" t="s">
+        <v>365</v>
+      </c>
+      <c r="G69" s="98" t="s">
         <v>363</v>
-      </c>
-      <c r="F69" s="126" t="s">
-        <v>366</v>
-      </c>
-      <c r="G69" s="98" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.3">
@@ -4203,19 +4231,19 @@
         <v>51</v>
       </c>
       <c r="C70" s="57" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="D70" s="58">
         <v>1</v>
       </c>
       <c r="E70" s="126" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="F70" s="126" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="G70" s="98" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.3">
@@ -4224,19 +4252,19 @@
         <v>52</v>
       </c>
       <c r="C71" s="57" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D71" s="56">
         <v>1</v>
       </c>
       <c r="E71" s="57" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F71" s="59" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G71" s="90" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.3">
@@ -4245,7 +4273,7 @@
         <v>53</v>
       </c>
       <c r="C72" s="57" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D72" s="58">
         <v>4</v>
@@ -4254,10 +4282,10 @@
         <v>57</v>
       </c>
       <c r="F72" s="59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G72" s="90" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.3">
@@ -4266,19 +4294,19 @@
         <v>54</v>
       </c>
       <c r="C73" s="72" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D73" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E73" s="74" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F73" s="74" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G73" s="98" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="74" spans="2:7" x14ac:dyDescent="0.3">
@@ -4287,7 +4315,7 @@
         <v>55</v>
       </c>
       <c r="C74" s="57" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D74" s="58">
         <v>3</v>
@@ -4296,10 +4324,10 @@
         <v>57</v>
       </c>
       <c r="F74" s="59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G74" s="90" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="75" spans="2:7" x14ac:dyDescent="0.3">
@@ -4308,7 +4336,7 @@
         <v>56</v>
       </c>
       <c r="C75" s="57" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D75" s="58">
         <v>1</v>
@@ -4317,10 +4345,10 @@
         <v>57</v>
       </c>
       <c r="F75" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G75" s="90" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="76" spans="2:7" x14ac:dyDescent="0.3">
@@ -4329,7 +4357,7 @@
         <v>57</v>
       </c>
       <c r="C76" s="57" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D76" s="58">
         <v>1</v>
@@ -4341,7 +4369,7 @@
         <v>62</v>
       </c>
       <c r="G76" s="90" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="77" spans="2:7" x14ac:dyDescent="0.3">
@@ -4350,7 +4378,7 @@
         <v>58</v>
       </c>
       <c r="C77" s="57" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D77" s="55" t="s">
         <v>56</v>
@@ -4371,7 +4399,7 @@
         <v>59</v>
       </c>
       <c r="C78" s="57" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D78" s="58">
         <v>6</v>
@@ -4380,10 +4408,10 @@
         <v>43</v>
       </c>
       <c r="F78" s="71" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G78" s="90" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="79" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -4392,7 +4420,7 @@
         <v>60</v>
       </c>
       <c r="C79" s="61" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D79" s="60" t="s">
         <v>44</v>
@@ -4413,7 +4441,7 @@
         <v>61</v>
       </c>
       <c r="C80" s="57" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D80" s="55" t="s">
         <v>54</v>
@@ -4434,7 +4462,7 @@
         <v>62</v>
       </c>
       <c r="C81" s="57" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D81" s="55" t="s">
         <v>55</v>
@@ -4446,7 +4474,7 @@
         <v>62</v>
       </c>
       <c r="G81" s="90" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="82" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -4455,7 +4483,7 @@
         <v>63</v>
       </c>
       <c r="C82" s="57" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D82" s="55" t="s">
         <v>55</v>
@@ -4464,10 +4492,10 @@
         <v>43</v>
       </c>
       <c r="F82" s="71" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G82" s="90" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="83" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
@@ -4476,7 +4504,7 @@
         <v>64</v>
       </c>
       <c r="C83" s="57" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D83" s="55" t="s">
         <v>55</v>
@@ -4485,10 +4513,10 @@
         <v>43</v>
       </c>
       <c r="F83" s="71" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="G83" s="90" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.3">
@@ -4497,7 +4525,7 @@
         <v>65</v>
       </c>
       <c r="C84" s="57" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D84" s="58">
         <v>5</v>
@@ -4518,19 +4546,19 @@
         <v>66</v>
       </c>
       <c r="C85" s="57" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D85" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E85" s="57" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F85" s="59" t="s">
         <v>43</v>
       </c>
       <c r="G85" s="90" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.3">
@@ -4539,7 +4567,7 @@
         <v>67</v>
       </c>
       <c r="C86" s="57" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D86" s="58">
         <v>2</v>
@@ -4548,10 +4576,10 @@
         <v>57</v>
       </c>
       <c r="F86" s="59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G86" s="90" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="87" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -4560,19 +4588,19 @@
         <v>68</v>
       </c>
       <c r="C87" s="57" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D87" s="60" t="s">
         <v>20</v>
       </c>
       <c r="E87" s="74" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F87" s="59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G87" s="90" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="88" spans="2:7" x14ac:dyDescent="0.3">
@@ -4581,19 +4609,19 @@
         <v>69</v>
       </c>
       <c r="C88" s="72" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D88" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E88" s="74" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="F88" s="74" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G88" s="98" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="89" spans="2:7" x14ac:dyDescent="0.3">
@@ -4602,7 +4630,7 @@
         <v>70</v>
       </c>
       <c r="C89" s="57" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D89" s="58">
         <v>1</v>
@@ -4611,10 +4639,10 @@
         <v>57</v>
       </c>
       <c r="F89" s="62" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G89" s="90" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="90" spans="2:7" x14ac:dyDescent="0.3">
@@ -4623,19 +4651,19 @@
         <v>71</v>
       </c>
       <c r="C90" s="57" t="s">
+        <v>256</v>
+      </c>
+      <c r="D90" s="55" t="s">
         <v>257</v>
       </c>
-      <c r="D90" s="55" t="s">
+      <c r="E90" s="57" t="s">
         <v>258</v>
       </c>
-      <c r="E90" s="57" t="s">
+      <c r="F90" s="59" t="s">
         <v>259</v>
       </c>
-      <c r="F90" s="59" t="s">
+      <c r="G90" s="90" t="s">
         <v>260</v>
-      </c>
-      <c r="G90" s="90" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.3">
@@ -4644,7 +4672,7 @@
         <v>72</v>
       </c>
       <c r="C91" s="57" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D91" s="58">
         <v>1</v>
@@ -4653,10 +4681,10 @@
         <v>57</v>
       </c>
       <c r="F91" s="59" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G91" s="90" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="92" spans="2:7" x14ac:dyDescent="0.3">
@@ -4665,7 +4693,7 @@
         <v>73</v>
       </c>
       <c r="C92" s="57" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D92" s="58">
         <v>1</v>
@@ -4674,10 +4702,10 @@
         <v>57</v>
       </c>
       <c r="F92" s="62" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G92" s="90" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.3">
@@ -4686,19 +4714,19 @@
         <v>74</v>
       </c>
       <c r="C93" s="57" t="s">
+        <v>261</v>
+      </c>
+      <c r="D93" s="55" t="s">
+        <v>257</v>
+      </c>
+      <c r="E93" s="57" t="s">
+        <v>258</v>
+      </c>
+      <c r="F93" s="59" t="s">
         <v>262</v>
       </c>
-      <c r="D93" s="55" t="s">
-        <v>258</v>
-      </c>
-      <c r="E93" s="57" t="s">
-        <v>259</v>
-      </c>
-      <c r="F93" s="59" t="s">
+      <c r="G93" s="90" t="s">
         <v>263</v>
-      </c>
-      <c r="G93" s="90" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="94" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -4707,19 +4735,19 @@
         <v>75</v>
       </c>
       <c r="C94" s="57" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D94" s="55" t="s">
         <v>20</v>
       </c>
       <c r="E94" s="57" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F94" s="71" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G94" s="91" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="95" spans="2:7" x14ac:dyDescent="0.3">
@@ -4728,7 +4756,7 @@
         <v>76</v>
       </c>
       <c r="C95" s="57" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D95" s="55" t="s">
         <v>19</v>
@@ -4737,10 +4765,10 @@
         <v>61</v>
       </c>
       <c r="F95" s="63" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G95" s="90" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.3">
@@ -4749,7 +4777,7 @@
         <v>77</v>
       </c>
       <c r="C96" s="63" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D96" s="64" t="s">
         <v>19</v>
@@ -4758,10 +4786,10 @@
         <v>61</v>
       </c>
       <c r="F96" s="63" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G96" s="93" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="97" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -4770,19 +4798,19 @@
         <v>78</v>
       </c>
       <c r="C97" s="72" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D97" s="55" t="s">
+        <v>292</v>
+      </c>
+      <c r="E97" s="74" t="s">
         <v>293</v>
       </c>
-      <c r="E97" s="74" t="s">
+      <c r="F97" s="74" t="s">
         <v>294</v>
       </c>
-      <c r="F97" s="74" t="s">
-        <v>295</v>
-      </c>
       <c r="G97" s="98" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="98" spans="2:7" x14ac:dyDescent="0.3">
@@ -4791,7 +4819,7 @@
         <v>79</v>
       </c>
       <c r="C98" s="57" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D98" s="58">
         <v>1</v>
@@ -4800,10 +4828,10 @@
         <v>57</v>
       </c>
       <c r="F98" s="59" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="G98" s="90" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="99" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -4812,7 +4840,7 @@
         <v>80</v>
       </c>
       <c r="C99" s="57" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D99" s="60" t="s">
         <v>45</v>
@@ -4821,7 +4849,7 @@
         <v>41</v>
       </c>
       <c r="F99" s="59" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="G99" s="90" t="s">
         <v>50</v>
@@ -4833,7 +4861,7 @@
         <v>81</v>
       </c>
       <c r="C100" s="57" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D100" s="58">
         <v>1</v>
@@ -4845,7 +4873,7 @@
         <v>42</v>
       </c>
       <c r="G100" s="90" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="101" spans="2:7" x14ac:dyDescent="0.3">
@@ -4854,7 +4882,7 @@
         <v>82</v>
       </c>
       <c r="C101" s="57" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D101" s="55" t="s">
         <v>19</v>
@@ -4863,10 +4891,10 @@
         <v>42</v>
       </c>
       <c r="F101" s="71" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="G101" s="90" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.3">
@@ -4875,7 +4903,7 @@
         <v>83</v>
       </c>
       <c r="C102" s="61" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D102" s="55" t="s">
         <v>20</v>
@@ -4884,10 +4912,10 @@
         <v>38</v>
       </c>
       <c r="F102" s="78" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G102" s="91" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="103" spans="2:7" x14ac:dyDescent="0.3">
@@ -4896,13 +4924,13 @@
         <v>84</v>
       </c>
       <c r="C103" s="65" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D103" s="12" t="s">
         <v>20</v>
       </c>
       <c r="E103" s="65" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F103" s="80" t="s">
         <v>11</v>
@@ -4917,7 +4945,7 @@
         <v>85</v>
       </c>
       <c r="C104" s="66" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D104" s="67">
         <v>1</v>
@@ -4938,7 +4966,7 @@
         <v>86</v>
       </c>
       <c r="C105" s="61" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D105" s="55" t="s">
         <v>20</v>
@@ -4947,10 +4975,10 @@
         <v>34</v>
       </c>
       <c r="F105" s="78" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="G105" s="91" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="106" spans="2:7" x14ac:dyDescent="0.3">
@@ -4959,19 +4987,19 @@
         <v>87</v>
       </c>
       <c r="C106" s="57" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D106" s="55" t="s">
         <v>20</v>
       </c>
       <c r="E106" s="57" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F106" s="59" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="G106" s="90" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="107" spans="2:7" x14ac:dyDescent="0.3">
@@ -4980,19 +5008,19 @@
         <v>88</v>
       </c>
       <c r="C107" s="57" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D107" s="55" t="s">
         <v>20</v>
       </c>
       <c r="E107" s="57" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F107" s="59" t="s">
         <v>34</v>
       </c>
       <c r="G107" s="90" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.3">
@@ -5001,19 +5029,19 @@
         <v>89</v>
       </c>
       <c r="C108" s="57" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="D108" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E108" s="126" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="F108" s="126" t="s">
         <v>35</v>
       </c>
       <c r="G108" s="98" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="109" spans="2:7" ht="66" x14ac:dyDescent="0.3">
@@ -5022,19 +5050,19 @@
         <v>90</v>
       </c>
       <c r="C109" s="57" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D109" s="58">
         <v>1</v>
       </c>
       <c r="E109" s="57" t="s">
+        <v>226</v>
+      </c>
+      <c r="F109" s="71" t="s">
+        <v>250</v>
+      </c>
+      <c r="G109" s="90" t="s">
         <v>227</v>
-      </c>
-      <c r="F109" s="71" t="s">
-        <v>251</v>
-      </c>
-      <c r="G109" s="90" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="110" spans="2:7" ht="82.5" x14ac:dyDescent="0.3">
@@ -5043,19 +5071,19 @@
         <v>91</v>
       </c>
       <c r="C110" s="68" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D110" s="18" t="s">
         <v>19</v>
       </c>
       <c r="E110" s="68" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F110" s="81" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="G110" s="96" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="111" spans="2:7" x14ac:dyDescent="0.3">
@@ -5064,19 +5092,19 @@
         <v>92</v>
       </c>
       <c r="C111" s="75" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D111" s="76" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E111" s="85" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F111" s="86" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G111" s="99" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="112" spans="2:7" x14ac:dyDescent="0.3">
@@ -5085,19 +5113,19 @@
         <v>93</v>
       </c>
       <c r="C112" s="72" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D112" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E112" s="74" t="s">
+        <v>264</v>
+      </c>
+      <c r="F112" s="74" t="s">
         <v>265</v>
       </c>
-      <c r="F112" s="74" t="s">
-        <v>266</v>
-      </c>
       <c r="G112" s="98" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="113" spans="2:7" x14ac:dyDescent="0.3">
@@ -5106,19 +5134,19 @@
         <v>94</v>
       </c>
       <c r="C113" s="57" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D113" s="55" t="s">
         <v>55</v>
       </c>
       <c r="E113" s="71" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F113" s="71" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G113" s="90" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="114" spans="2:7" x14ac:dyDescent="0.3">
@@ -5127,19 +5155,19 @@
         <v>95</v>
       </c>
       <c r="C114" s="57" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D114" s="58">
         <v>1</v>
       </c>
       <c r="E114" s="59" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F114" s="71" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G114" s="90" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="115" spans="2:7" x14ac:dyDescent="0.3">
@@ -5148,19 +5176,19 @@
         <v>96</v>
       </c>
       <c r="C115" s="57" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D115" s="58">
         <v>2</v>
       </c>
       <c r="E115" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="F115" s="59" t="s">
         <v>119</v>
       </c>
-      <c r="F115" s="59" t="s">
-        <v>120</v>
-      </c>
       <c r="G115" s="90" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="116" spans="2:7" x14ac:dyDescent="0.3">
@@ -5169,19 +5197,19 @@
         <v>97</v>
       </c>
       <c r="C116" s="72" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D116" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E116" s="74" t="s">
+        <v>264</v>
+      </c>
+      <c r="F116" s="74" t="s">
         <v>265</v>
       </c>
-      <c r="F116" s="74" t="s">
-        <v>266</v>
-      </c>
       <c r="G116" s="98" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="117" spans="2:7" x14ac:dyDescent="0.3">
@@ -5190,19 +5218,19 @@
         <v>98</v>
       </c>
       <c r="C117" s="68" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D117" s="69">
         <v>1</v>
       </c>
       <c r="E117" s="68" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F117" s="82" t="s">
         <v>13</v>
       </c>
       <c r="G117" s="96" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="118" spans="2:7" x14ac:dyDescent="0.3">
@@ -5211,19 +5239,19 @@
         <v>99</v>
       </c>
       <c r="C118" s="72" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D118" s="55" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E118" s="74" t="s">
+        <v>264</v>
+      </c>
+      <c r="F118" s="74" t="s">
         <v>265</v>
       </c>
-      <c r="F118" s="74" t="s">
-        <v>266</v>
-      </c>
       <c r="G118" s="98" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="119" spans="2:7" x14ac:dyDescent="0.3">
@@ -5232,40 +5260,40 @@
         <v>100</v>
       </c>
       <c r="C119" s="57" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D119" s="58">
         <v>1</v>
       </c>
       <c r="E119" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="F119" s="59" t="s">
         <v>119</v>
       </c>
-      <c r="F119" s="59" t="s">
-        <v>120</v>
-      </c>
       <c r="G119" s="90" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="120" spans="2:7" ht="33" x14ac:dyDescent="0.3">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="120" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
       <c r="B120" s="89">
         <f t="shared" si="3"/>
         <v>101</v>
       </c>
       <c r="C120" s="68" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D120" s="69">
         <v>1</v>
       </c>
       <c r="E120" s="68" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F120" s="83" t="s">
-        <v>64</v>
+        <v>379</v>
       </c>
       <c r="G120" s="96" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="121" spans="2:7" x14ac:dyDescent="0.3">
@@ -5274,19 +5302,19 @@
         <v>102</v>
       </c>
       <c r="C121" s="77" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D121" s="18" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E121" s="87" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F121" s="88" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="G121" s="100" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="122" spans="2:7" x14ac:dyDescent="0.3">
@@ -5295,19 +5323,19 @@
         <v>103</v>
       </c>
       <c r="C122" s="57" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D122" s="55" t="s">
         <v>20</v>
       </c>
       <c r="E122" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="F122" s="59" t="s">
         <v>119</v>
       </c>
-      <c r="F122" s="59" t="s">
-        <v>120</v>
-      </c>
       <c r="G122" s="90" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="123" spans="2:7" x14ac:dyDescent="0.3">
@@ -5316,19 +5344,19 @@
         <v>104</v>
       </c>
       <c r="C123" s="63" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D123" s="64" t="s">
         <v>19</v>
       </c>
       <c r="E123" s="63" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F123" s="84" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G123" s="93" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="124" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -5337,19 +5365,19 @@
         <v>105</v>
       </c>
       <c r="C124" s="57" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D124" s="55" t="s">
         <v>55</v>
       </c>
       <c r="E124" s="57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F124" s="71" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="G124" s="90" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="125" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -5358,19 +5386,19 @@
         <v>106</v>
       </c>
       <c r="C125" s="57" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D125" s="58">
         <v>1</v>
       </c>
       <c r="E125" s="59" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F125" s="71" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="G125" s="90" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="126" spans="2:7" x14ac:dyDescent="0.3">
@@ -5379,19 +5407,19 @@
         <v>107</v>
       </c>
       <c r="C126" s="68" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D126" s="18" t="s">
         <v>19</v>
       </c>
       <c r="E126" s="70" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F126" s="82" t="s">
         <v>16</v>
       </c>
       <c r="G126" s="96" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="127" spans="2:7" x14ac:dyDescent="0.3">
@@ -5400,19 +5428,19 @@
         <v>108</v>
       </c>
       <c r="C127" s="57" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D127" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E127" s="57" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F127" s="57" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G127" s="90" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="128" spans="2:7" ht="49.5" x14ac:dyDescent="0.3">
@@ -5421,19 +5449,19 @@
         <v>109</v>
       </c>
       <c r="C128" s="57" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D128" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E128" s="57" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F128" s="71" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="G128" s="90" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="129" spans="2:7" x14ac:dyDescent="0.3">
@@ -5442,19 +5470,19 @@
         <v>110</v>
       </c>
       <c r="C129" s="72" t="s">
+        <v>281</v>
+      </c>
+      <c r="D129" s="58" t="s">
+        <v>286</v>
+      </c>
+      <c r="E129" s="74" t="s">
+        <v>265</v>
+      </c>
+      <c r="F129" s="74" t="s">
         <v>282</v>
       </c>
-      <c r="D129" s="58" t="s">
-        <v>287</v>
-      </c>
-      <c r="E129" s="74" t="s">
-        <v>266</v>
-      </c>
-      <c r="F129" s="74" t="s">
-        <v>283</v>
-      </c>
       <c r="G129" s="98" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="130" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -5463,19 +5491,19 @@
         <v>111</v>
       </c>
       <c r="C130" s="72" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D130" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E130" s="74" t="s">
+        <v>297</v>
+      </c>
+      <c r="F130" s="74" t="s">
         <v>298</v>
       </c>
-      <c r="F130" s="74" t="s">
-        <v>299</v>
-      </c>
       <c r="G130" s="98" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="131" spans="2:7" x14ac:dyDescent="0.3">
@@ -5484,19 +5512,19 @@
         <v>112</v>
       </c>
       <c r="C131" s="57" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D131" s="58">
         <v>1</v>
       </c>
       <c r="E131" s="59" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F131" s="59" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G131" s="90" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="132" spans="2:7" x14ac:dyDescent="0.3">
@@ -5505,19 +5533,19 @@
         <v>113</v>
       </c>
       <c r="C132" s="72" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D132" s="55" t="s">
+        <v>299</v>
+      </c>
+      <c r="E132" s="74" t="s">
         <v>300</v>
       </c>
-      <c r="E132" s="74" t="s">
+      <c r="F132" s="74" t="s">
         <v>301</v>
       </c>
-      <c r="F132" s="74" t="s">
-        <v>302</v>
-      </c>
       <c r="G132" s="98" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="133" spans="2:7" ht="33" x14ac:dyDescent="0.3">
@@ -5526,19 +5554,19 @@
         <v>114</v>
       </c>
       <c r="C133" s="57" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D133" s="58">
         <v>2</v>
       </c>
       <c r="E133" s="59" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F133" s="71" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G133" s="90" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="134" spans="2:7" x14ac:dyDescent="0.3">
@@ -5547,19 +5575,19 @@
         <v>115</v>
       </c>
       <c r="C134" s="72" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D134" s="58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="E134" s="74" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F134" s="74" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G134" s="98" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="135" spans="2:7" x14ac:dyDescent="0.3">
@@ -5568,19 +5596,19 @@
         <v>116</v>
       </c>
       <c r="C135" s="72" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D135" s="55" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E135" s="74" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F135" s="74" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G135" s="98" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="136" spans="2:7" ht="66" x14ac:dyDescent="0.3">
@@ -5589,19 +5617,19 @@
         <v>117</v>
       </c>
       <c r="C136" s="57" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D136" s="55" t="s">
         <v>19</v>
       </c>
       <c r="E136" s="57" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F136" s="71" t="s">
+        <v>368</v>
+      </c>
+      <c r="G136" s="90" t="s">
         <v>369</v>
-      </c>
-      <c r="G136" s="90" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="137" spans="2:7" x14ac:dyDescent="0.3">
@@ -5610,19 +5638,19 @@
         <v>118</v>
       </c>
       <c r="C137" s="122" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D137" s="127" t="s">
         <v>20</v>
       </c>
       <c r="E137" s="123" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F137" s="124" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G137" s="125" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="138" spans="2:7" x14ac:dyDescent="0.3">
@@ -5631,19 +5659,19 @@
         <v>119</v>
       </c>
       <c r="C138" s="57" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D138" s="55" t="s">
         <v>55</v>
       </c>
       <c r="E138" s="59" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F138" s="71" t="s">
         <v>61</v>
       </c>
       <c r="G138" s="90" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="139" spans="2:7" ht="66" x14ac:dyDescent="0.3">
@@ -5652,19 +5680,19 @@
         <v>120</v>
       </c>
       <c r="C139" s="57" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D139" s="55" t="s">
         <v>55</v>
       </c>
       <c r="E139" s="57" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F139" s="71" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="G139" s="90" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="140" spans="2:7" ht="66.75" thickBot="1" x14ac:dyDescent="0.35">
@@ -5673,19 +5701,19 @@
         <v>121</v>
       </c>
       <c r="C140" s="116" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D140" s="117">
         <v>1</v>
       </c>
       <c r="E140" s="118" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F140" s="119" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="G140" s="120" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="141" spans="2:7" x14ac:dyDescent="0.3">

</xml_diff>